<commit_message>
feat(tts): word-by-word highlight sync, loading spinner, threat model closeout
- Switch to textToSpeechWithTimestamps for character alignment
- Replace ontimeupdate with requestAnimationFrame for frame-rate word tracking
- Binary search over word ranges per RAF tick
- Fix word endTime to use next word startTime eliminating inter-word gaps
- Add loading AudioState with spinning ribbon icon during API call
- Guard command palette from loading state re-entrancy
- Fix selectedModelId null bug on Settings display
- DEFAULT_MODEL_ID fallback so null model never blocks playback
- Reset state and ribbon to idle on error and non-200 responses
- stopRAF called on onended and onunload
- T1 accepted, T3 false-positive, T8 false-positive in threat model
- Regenerated all threagile docs
- Updated README with per-risk findings
- Bump version to 2.2.0
</commit_message>
<xml_diff>
--- a/docs/risks.xlsx
+++ b/docs/risks.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
   <si>
     <t>Severity</t>
   </si>
@@ -118,13 +118,13 @@
     <t>t1-api-key-plaintext-data-json@obsidian-vault-storage@local-user-workstation@elevenlabs-api-key</t>
   </si>
   <si>
-    <t>in Progress</t>
-  </si>
-  <si>
-    <t>Migration from plaintext `data.json` secret storage to safer storage is in progress.</t>
-  </si>
-  <si>
-    <t>2026-03-09</t>
+    <t>Accepted</t>
+  </si>
+  <si>
+    <t>saveData() serialises apiKey into data.json as a plain string. The Obsidian platform provides no secret store, so plaintext persistence is an unavoidable platform constraint. A security notice is displayed to the user in the settings tab (src/settings.ts). No code change can fully mitigate this within the plugin model; documented as accepted risk.</t>
+  </si>
+  <si>
+    <t>2026-04-03</t>
   </si>
   <si>
     <t>vonst</t>
@@ -133,21 +133,282 @@
     <t>T1</t>
   </si>
   <si>
+    <t>Elevated</t>
+  </si>
+  <si>
+    <t>Unlikely</t>
+  </si>
+  <si>
+    <t>Very High</t>
+  </si>
+  <si>
     <t>Tampering</t>
   </si>
   <si>
+    <t>Operations</t>
+  </si>
+  <si>
+    <t>CWE-1008</t>
+  </si>
+  <si>
+    <t>Missing Cloud Hardening</t>
+  </si>
+  <si>
+    <t>Missing Cloud Hardening risk at ElevenLabs Cloud</t>
+  </si>
+  <si>
+    <t>Cloud Hardening</t>
+  </si>
+  <si>
+    <t>Apply hardening of all cloud components and services, taking special care to follow the individual risk descriptions (which depend on the cloud provider tags in the model). &lt;br&gt;&lt;br&gt;For &lt;b&gt;Amazon Web Services (AWS)&lt;/b&gt;: Follow the &lt;i&gt;CIS Benchmark for Amazon Web Services&lt;/i&gt; (see also the automated checks of cloud audit tools like &lt;i&gt;"PacBot", "CloudSploit", "CloudMapper", "ScoutSuite", or "Prowler AWS CIS Benchmark Tool"&lt;/i&gt;). &lt;br&gt;For EC2 and other servers running Amazon Linux, follow the &lt;i&gt;CIS Benchmark for Amazon Linux&lt;/i&gt; and switch to IMDSv2. &lt;br&gt;For S3 buckets follow the &lt;i&gt;Security Best Practices for Amazon S3&lt;/i&gt; at &lt;a href="https://docs.aws.amazon.com/AmazonS3/latest/dev/security-best-practices.html"&gt;https://docs.aws.amazon.com/AmazonS3/latest/dev/security-best-practices.html&lt;/a&gt; to avoid accidental leakage. &lt;br&gt;Also take a look at some of these tools: &lt;a href="https://github.com/toniblyx/my-arsenal-of-aws-security-tools"&gt;https://github.com/toniblyx/my-arsenal-of-aws-security-tools&lt;/a&gt; &lt;br&gt;&lt;br&gt;For &lt;b&gt;Microsoft Azure&lt;/b&gt;: Follow the &lt;i&gt;CIS Benchmark for Microsoft Azure&lt;/i&gt; (see also the automated checks of cloud audit tools like &lt;i&gt;"CloudSploit" or "ScoutSuite"&lt;/i&gt;).&lt;br&gt;&lt;br&gt;For &lt;b&gt;Google Cloud Platform&lt;/b&gt;: Follow the &lt;i&gt;CIS Benchmark for Google Cloud Computing Platform&lt;/i&gt; (see also the automated checks of cloud audit tools like &lt;i&gt;"CloudSploit" or "ScoutSuite"&lt;/i&gt;). &lt;br&gt;&lt;br&gt;For &lt;b&gt;Oracle Cloud Platform&lt;/b&gt;: Follow the hardening best practices (see also the automated checks of cloud audit tools like &lt;i&gt;"CloudSploit"&lt;/i&gt;).</t>
+  </si>
+  <si>
+    <t>Are recommendations from the linked cheat sheet and referenced ASVS chapter applied?</t>
+  </si>
+  <si>
+    <t>missing-cloud-hardening@elevenlabs-cloud</t>
+  </si>
+  <si>
+    <t>Unchecked</t>
+  </si>
+  <si>
+    <t>Very Likely</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Spoofing</t>
+  </si>
+  <si>
     <t>Development</t>
   </si>
   <si>
+    <t>CWE-434</t>
+  </si>
+  <si>
+    <t>Missing File Validation</t>
+  </si>
+  <si>
+    <t>Obsidian Plugin Runtime</t>
+  </si>
+  <si>
+    <t>Missing File Validation risk at Obsidian Plugin Runtime</t>
+  </si>
+  <si>
+    <t>File Validation</t>
+  </si>
+  <si>
+    <t>Filter by file extension and discard (if feasible) the name provided. Whitelist the accepted file types and determine the mime-type on the server-side (for example via "Apache Tika" or similar checks). If the file is retrievable by endusers and/or backoffice employees, consider performing scans for popular malware (if the files can be retrieved much later than they were uploaded, also apply a fresh malware scan during retrieval to scan with newer signatures of popular malware). Also enforce limits on maximum file size to avoid denial-of-service like scenarios.</t>
+  </si>
+  <si>
+    <t>missing-file-validation@obsidian-plugin-runtime</t>
+  </si>
+  <si>
+    <t>CWE-16</t>
+  </si>
+  <si>
+    <t>Missing Hardening</t>
+  </si>
+  <si>
+    <t>Missing Hardening risk at Obsidian Vault Storage</t>
+  </si>
+  <si>
+    <t>System Hardening</t>
+  </si>
+  <si>
+    <t>Try to apply all hardening best practices (like CIS benchmarks, OWASP recommendations, vendor recommendations, DevSec Hardening Framework, DBSAT for Oracle databases, and others).</t>
+  </si>
+  <si>
+    <t>missing-hardening@obsidian-vault-storage</t>
+  </si>
+  <si>
     <t>CWE-22</t>
   </si>
   <si>
+    <t>Path-Traversal</t>
+  </si>
+  <si>
+    <t>Read or Write Vault Files</t>
+  </si>
+  <si>
+    <t>Path-Traversal risk at Obsidian Plugin Runtime against filesystem Obsidian Vault Storage via Read or Write Vault Files</t>
+  </si>
+  <si>
+    <t>Path-Traversal Prevention</t>
+  </si>
+  <si>
+    <t>Before accessing the file cross-check that it resides in the expected folder and is of the expected type and filename/suffix. Try to use a mapping if possible instead of directly accessing by a filename which is (partly or fully) provided by the caller. When a third-party product is used instead of custom developed software, check if the product applies the proper mitigation and ensure a reasonable patch-level.</t>
+  </si>
+  <si>
+    <t>path-traversal@obsidian-plugin-runtime@obsidian-vault-storage@obsidian-plugin-runtime&gt;read-or-write-vault-files</t>
+  </si>
+  <si>
+    <t>Elevation of Privilege</t>
+  </si>
+  <si>
+    <t>CWE-501</t>
+  </si>
+  <si>
+    <t>Unguarded Access From Internet</t>
+  </si>
+  <si>
+    <t>Unguarded Access from Internet of Obsidian Vault Storage by Obsidian Plugin Runtime via Read or Write Vault Files</t>
+  </si>
+  <si>
+    <t>Encapsulation of Technical Asset</t>
+  </si>
+  <si>
+    <t>Encapsulate the asset behind a guarding service, application, or reverse-proxy. For admin maintenance a bastion-host should be used as a jump-server. For file transfer a store-and-forward-host should be used as an indirect file exchange platform.</t>
+  </si>
+  <si>
+    <t>unguarded-access-from-internet@obsidian-vault-storage@obsidian-plugin-runtime@obsidian-plugin-runtime&gt;read-or-write-vault-files</t>
+  </si>
+  <si>
+    <t>CWE-1127</t>
+  </si>
+  <si>
+    <t>Missing Build Infrastructure</t>
+  </si>
+  <si>
+    <t>Missing Build Infrastructure in the threat model (referencing asset Obsidian Plugin Runtime as an example)</t>
+  </si>
+  <si>
+    <t>Build Pipeline Hardening</t>
+  </si>
+  <si>
+    <t>Include the build infrastructure in the model.</t>
+  </si>
+  <si>
+    <t>missing-build-infrastructure@obsidian-plugin-runtime</t>
+  </si>
+  <si>
+    <t>CWE-287</t>
+  </si>
+  <si>
+    <t>Missing Identity Store</t>
+  </si>
+  <si>
+    <t>Missing Identity Store in the threat model (referencing asset Obsidian Plugin Runtime as an example)</t>
+  </si>
+  <si>
+    <t>Identity Store</t>
+  </si>
+  <si>
+    <t>Include an identity store in the model if the application has a login.</t>
+  </si>
+  <si>
+    <t>missing-identity-store@obsidian-plugin-runtime</t>
+  </si>
+  <si>
+    <t>Missing Network Segmentation</t>
+  </si>
+  <si>
+    <t>Missing Network Segmentation to further encapsulate and protect Obsidian Vault Storage against unrelated lower protected assets in the same network segment, which might be easier to compromise by attackers</t>
+  </si>
+  <si>
+    <t>Network Segmentation</t>
+  </si>
+  <si>
+    <t>Apply a network segmentation trust-boundary around the highly sensitive assets and/or datastores.</t>
+  </si>
+  <si>
+    <t>missing-network-segmentation@obsidian-vault-storage</t>
+  </si>
+  <si>
+    <t>Business Side</t>
+  </si>
+  <si>
+    <t>CWE-308</t>
+  </si>
+  <si>
+    <t>Missing Two-Factor Authentication (2FA)</t>
+  </si>
+  <si>
+    <t>Trigger TTS Command</t>
+  </si>
+  <si>
+    <t>Missing Two-Factor Authentication covering communication link Trigger TTS Command from Obsidian End User to Obsidian Plugin Runtime</t>
+  </si>
+  <si>
+    <t>Authentication with Second Factor (2FA)</t>
+  </si>
+  <si>
+    <t>Apply an authentication method to the technical asset protecting highly sensitive data via two-factor authentication for human users.</t>
+  </si>
+  <si>
+    <t>missing-authentication-second-factor@obsidian-end-user&gt;trigger-tts-command@obsidian-end-user@obsidian-plugin-runtime</t>
+  </si>
+  <si>
+    <t>CWE-522</t>
+  </si>
+  <si>
+    <t>Missing Vault (Secret Storage)</t>
+  </si>
+  <si>
+    <t>Missing Vault (Secret Storage) in the threat model (referencing asset Obsidian Vault Storage as an example)</t>
+  </si>
+  <si>
+    <t>Vault (Secret Storage)</t>
+  </si>
+  <si>
+    <t>Consider using a Vault (Secret Storage) to securely store and access config secrets (like credentials, private keys, client certificates, etc.).</t>
+  </si>
+  <si>
+    <t>Is a Vault (Secret Storage) in place?</t>
+  </si>
+  <si>
+    <t>missing-vault@obsidian-vault-storage</t>
+  </si>
+  <si>
+    <t>CWE-311</t>
+  </si>
+  <si>
+    <t>Unencrypted Technical Assets</t>
+  </si>
+  <si>
+    <t>Unencrypted Technical Asset named Obsidian Plugin Runtime</t>
+  </si>
+  <si>
+    <t>Encryption of Technical Asset</t>
+  </si>
+  <si>
+    <t>Apply encryption to the technical asset.</t>
+  </si>
+  <si>
+    <t>unencrypted-asset@obsidian-plugin-runtime</t>
+  </si>
+  <si>
+    <t>Unencrypted Technical Asset named Obsidian Vault Storage missing enduser-individual encryption with data-with-enduser-individual-key</t>
+  </si>
+  <si>
+    <t>unencrypted-asset@obsidian-vault-storage</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Wrong Communication Link Content</t>
+  </si>
+  <si>
+    <t>Obsidian End User</t>
+  </si>
+  <si>
+    <t>Wrong Communication Link Content (protocol type "in-process-library-call" does not match target technology type "desktop": expected "library") at Obsidian End User regarding communication link Trigger TTS Command</t>
+  </si>
+  <si>
+    <t>Model Consistency</t>
+  </si>
+  <si>
+    <t>Try to model the correct readonly flag and/or data sent/received of communication links. Also try to use  communication link types matching the target technology/machine types.</t>
+  </si>
+  <si>
+    <t>wrong-communication-link-content@obsidian-end-user@obsidian-end-user&gt;trigger-tts-command</t>
+  </si>
+  <si>
     <t>T3 Audio Output Path Traversal</t>
   </si>
   <si>
-    <t>Obsidian Plugin Runtime</t>
-  </si>
-  <si>
     <t>Potential traversal in mp3 vault write path</t>
   </si>
   <si>
@@ -163,7 +424,10 @@
     <t>t3-audio-output-path-traversal@obsidian-plugin-runtime@local-user-workstation@generated-audio-files</t>
   </si>
   <si>
-    <t>Path canonicalization and vault-root enforcement are being implemented.</t>
+    <t>False Positive</t>
+  </si>
+  <si>
+    <t>createVaultDirectories (src/util/file.ts) and generateFilename are dead code — neither function is imported or called anywhere in the active codebase. No vault writes occur; audio plays entirely from an in-memory Blob URL (src/util/audio.ts). Path traversal via vault writes is not possible in the current implementation.</t>
   </si>
   <si>
     <t>T3</t>
@@ -190,265 +454,10 @@
     <t>t8-api-key-logging-leak@obsidian-plugin-runtime@local-user-workstation@elevenlabs-api-key</t>
   </si>
   <si>
-    <t>Unchecked</t>
-  </si>
-  <si>
-    <t>Elevated</t>
-  </si>
-  <si>
-    <t>Unlikely</t>
-  </si>
-  <si>
-    <t>Very High</t>
-  </si>
-  <si>
-    <t>Operations</t>
-  </si>
-  <si>
-    <t>CWE-1008</t>
-  </si>
-  <si>
-    <t>Missing Cloud Hardening</t>
-  </si>
-  <si>
-    <t>Missing Cloud Hardening risk at ElevenLabs Cloud</t>
-  </si>
-  <si>
-    <t>Cloud Hardening</t>
-  </si>
-  <si>
-    <t>Apply hardening of all cloud components and services, taking special care to follow the individual risk descriptions (which depend on the cloud provider tags in the model). &lt;br&gt;&lt;br&gt;For &lt;b&gt;Amazon Web Services (AWS)&lt;/b&gt;: Follow the &lt;i&gt;CIS Benchmark for Amazon Web Services&lt;/i&gt; (see also the automated checks of cloud audit tools like &lt;i&gt;"PacBot", "CloudSploit", "CloudMapper", "ScoutSuite", or "Prowler AWS CIS Benchmark Tool"&lt;/i&gt;). &lt;br&gt;For EC2 and other servers running Amazon Linux, follow the &lt;i&gt;CIS Benchmark for Amazon Linux&lt;/i&gt; and switch to IMDSv2. &lt;br&gt;For S3 buckets follow the &lt;i&gt;Security Best Practices for Amazon S3&lt;/i&gt; at &lt;a href="https://docs.aws.amazon.com/AmazonS3/latest/dev/security-best-practices.html"&gt;https://docs.aws.amazon.com/AmazonS3/latest/dev/security-best-practices.html&lt;/a&gt; to avoid accidental leakage. &lt;br&gt;Also take a look at some of these tools: &lt;a href="https://github.com/toniblyx/my-arsenal-of-aws-security-tools"&gt;https://github.com/toniblyx/my-arsenal-of-aws-security-tools&lt;/a&gt; &lt;br&gt;&lt;br&gt;For &lt;b&gt;Microsoft Azure&lt;/b&gt;: Follow the &lt;i&gt;CIS Benchmark for Microsoft Azure&lt;/i&gt; (see also the automated checks of cloud audit tools like &lt;i&gt;"CloudSploit" or "ScoutSuite"&lt;/i&gt;).&lt;br&gt;&lt;br&gt;For &lt;b&gt;Google Cloud Platform&lt;/b&gt;: Follow the &lt;i&gt;CIS Benchmark for Google Cloud Computing Platform&lt;/i&gt; (see also the automated checks of cloud audit tools like &lt;i&gt;"CloudSploit" or "ScoutSuite"&lt;/i&gt;). &lt;br&gt;&lt;br&gt;For &lt;b&gt;Oracle Cloud Platform&lt;/b&gt;: Follow the hardening best practices (see also the automated checks of cloud audit tools like &lt;i&gt;"CloudSploit"&lt;/i&gt;).</t>
-  </si>
-  <si>
-    <t>Are recommendations from the linked cheat sheet and referenced ASVS chapter applied?</t>
-  </si>
-  <si>
-    <t>missing-cloud-hardening@elevenlabs-cloud</t>
-  </si>
-  <si>
-    <t>Very Likely</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>Spoofing</t>
-  </si>
-  <si>
-    <t>CWE-434</t>
-  </si>
-  <si>
-    <t>Missing File Validation</t>
-  </si>
-  <si>
-    <t>Missing File Validation risk at Obsidian Plugin Runtime</t>
-  </si>
-  <si>
-    <t>File Validation</t>
-  </si>
-  <si>
-    <t>Filter by file extension and discard (if feasible) the name provided. Whitelist the accepted file types and determine the mime-type on the server-side (for example via "Apache Tika" or similar checks). If the file is retrievable by endusers and/or backoffice employees, consider performing scans for popular malware (if the files can be retrieved much later than they were uploaded, also apply a fresh malware scan during retrieval to scan with newer signatures of popular malware). Also enforce limits on maximum file size to avoid denial-of-service like scenarios.</t>
-  </si>
-  <si>
-    <t>missing-file-validation@obsidian-plugin-runtime</t>
-  </si>
-  <si>
-    <t>CWE-16</t>
-  </si>
-  <si>
-    <t>Missing Hardening</t>
-  </si>
-  <si>
-    <t>Missing Hardening risk at Obsidian Vault Storage</t>
-  </si>
-  <si>
-    <t>System Hardening</t>
-  </si>
-  <si>
-    <t>Try to apply all hardening best practices (like CIS benchmarks, OWASP recommendations, vendor recommendations, DevSec Hardening Framework, DBSAT for Oracle databases, and others).</t>
-  </si>
-  <si>
-    <t>missing-hardening@obsidian-vault-storage</t>
-  </si>
-  <si>
-    <t>Path-Traversal</t>
-  </si>
-  <si>
-    <t>Read or Write Vault Files</t>
-  </si>
-  <si>
-    <t>Path-Traversal risk at Obsidian Plugin Runtime against filesystem Obsidian Vault Storage via Read or Write Vault Files</t>
-  </si>
-  <si>
-    <t>Path-Traversal Prevention</t>
-  </si>
-  <si>
-    <t>Before accessing the file cross-check that it resides in the expected folder and is of the expected type and filename/suffix. Try to use a mapping if possible instead of directly accessing by a filename which is (partly or fully) provided by the caller. When a third-party product is used instead of custom developed software, check if the product applies the proper mitigation and ensure a reasonable patch-level.</t>
-  </si>
-  <si>
-    <t>path-traversal@obsidian-plugin-runtime@obsidian-vault-storage@obsidian-plugin-runtime&gt;read-or-write-vault-files</t>
-  </si>
-  <si>
-    <t>Elevation of Privilege</t>
-  </si>
-  <si>
-    <t>CWE-501</t>
-  </si>
-  <si>
-    <t>Unguarded Access From Internet</t>
-  </si>
-  <si>
-    <t>Unguarded Access from Internet of Obsidian Vault Storage by Obsidian Plugin Runtime via Read or Write Vault Files</t>
-  </si>
-  <si>
-    <t>Encapsulation of Technical Asset</t>
-  </si>
-  <si>
-    <t>Encapsulate the asset behind a guarding service, application, or reverse-proxy. For admin maintenance a bastion-host should be used as a jump-server. For file transfer a store-and-forward-host should be used as an indirect file exchange platform.</t>
-  </si>
-  <si>
-    <t>unguarded-access-from-internet@obsidian-vault-storage@obsidian-plugin-runtime@obsidian-plugin-runtime&gt;read-or-write-vault-files</t>
-  </si>
-  <si>
-    <t>CWE-1127</t>
-  </si>
-  <si>
-    <t>Missing Build Infrastructure</t>
-  </si>
-  <si>
-    <t>Missing Build Infrastructure in the threat model (referencing asset Obsidian Plugin Runtime as an example)</t>
-  </si>
-  <si>
-    <t>Build Pipeline Hardening</t>
-  </si>
-  <si>
-    <t>Include the build infrastructure in the model.</t>
-  </si>
-  <si>
-    <t>missing-build-infrastructure@obsidian-plugin-runtime</t>
-  </si>
-  <si>
-    <t>CWE-287</t>
-  </si>
-  <si>
-    <t>Missing Identity Store</t>
-  </si>
-  <si>
-    <t>Missing Identity Store in the threat model (referencing asset Obsidian Plugin Runtime as an example)</t>
-  </si>
-  <si>
-    <t>Identity Store</t>
-  </si>
-  <si>
-    <t>Include an identity store in the model if the application has a login.</t>
-  </si>
-  <si>
-    <t>missing-identity-store@obsidian-plugin-runtime</t>
-  </si>
-  <si>
-    <t>Missing Network Segmentation</t>
-  </si>
-  <si>
-    <t>Missing Network Segmentation to further encapsulate and protect Obsidian Vault Storage against unrelated lower protected assets in the same network segment, which might be easier to compromise by attackers</t>
-  </si>
-  <si>
-    <t>Network Segmentation</t>
-  </si>
-  <si>
-    <t>Apply a network segmentation trust-boundary around the highly sensitive assets and/or datastores.</t>
-  </si>
-  <si>
-    <t>missing-network-segmentation@obsidian-vault-storage</t>
-  </si>
-  <si>
-    <t>Business Side</t>
-  </si>
-  <si>
-    <t>CWE-308</t>
-  </si>
-  <si>
-    <t>Missing Two-Factor Authentication (2FA)</t>
-  </si>
-  <si>
-    <t>Trigger TTS Command</t>
-  </si>
-  <si>
-    <t>Missing Two-Factor Authentication covering communication link Trigger TTS Command from Obsidian End User to Obsidian Plugin Runtime</t>
-  </si>
-  <si>
-    <t>Authentication with Second Factor (2FA)</t>
-  </si>
-  <si>
-    <t>Apply an authentication method to the technical asset protecting highly sensitive data via two-factor authentication for human users.</t>
-  </si>
-  <si>
-    <t>missing-authentication-second-factor@obsidian-end-user&gt;trigger-tts-command@obsidian-end-user@obsidian-plugin-runtime</t>
-  </si>
-  <si>
-    <t>CWE-522</t>
-  </si>
-  <si>
-    <t>Missing Vault (Secret Storage)</t>
-  </si>
-  <si>
-    <t>Missing Vault (Secret Storage) in the threat model (referencing asset Obsidian Vault Storage as an example)</t>
-  </si>
-  <si>
-    <t>Vault (Secret Storage)</t>
-  </si>
-  <si>
-    <t>Consider using a Vault (Secret Storage) to securely store and access config secrets (like credentials, private keys, client certificates, etc.).</t>
-  </si>
-  <si>
-    <t>Is a Vault (Secret Storage) in place?</t>
-  </si>
-  <si>
-    <t>missing-vault@obsidian-vault-storage</t>
-  </si>
-  <si>
-    <t>CWE-311</t>
-  </si>
-  <si>
-    <t>Unencrypted Technical Assets</t>
-  </si>
-  <si>
-    <t>Unencrypted Technical Asset named Obsidian Plugin Runtime</t>
-  </si>
-  <si>
-    <t>Encryption of Technical Asset</t>
-  </si>
-  <si>
-    <t>Apply encryption to the technical asset.</t>
-  </si>
-  <si>
-    <t>unencrypted-asset@obsidian-plugin-runtime</t>
-  </si>
-  <si>
-    <t>Unencrypted Technical Asset named Obsidian Vault Storage missing enduser-individual encryption with data-with-enduser-individual-key</t>
-  </si>
-  <si>
-    <t>unencrypted-asset@obsidian-vault-storage</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>Wrong Communication Link Content</t>
-  </si>
-  <si>
-    <t>Obsidian End User</t>
-  </si>
-  <si>
-    <t>Wrong Communication Link Content (protocol type "in-process-library-call" does not match target technology type "desktop": expected "library") at Obsidian End User regarding communication link Trigger TTS Command</t>
-  </si>
-  <si>
-    <t>Model Consistency</t>
-  </si>
-  <si>
-    <t>Try to model the correct readonly flag and/or data sent/received of communication links. Also try to use  communication link types matching the target technology/machine types.</t>
-  </si>
-  <si>
-    <t>wrong-communication-link-content@obsidian-end-user@obsidian-end-user&gt;trigger-tts-command</t>
+    <t>There are no console.log calls anywhere in the project. All logging uses console.error and none of those call sites include this.secrets.apiKey or any request headers — only generic status messages and caught error objects are logged. Confirmed clean.</t>
+  </si>
+  <si>
+    <t>T8</t>
   </si>
 </sst>
 </file>
@@ -1087,7 +1096,7 @@
       <c r="O2" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="P2" s="12" t="s">
+      <c r="P2" s="13" t="s">
         <v>34</v>
       </c>
       <c r="Q2" s="19" t="s">
@@ -1104,115 +1113,107 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="A3" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="B3" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="C3" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="D3" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="E3" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="F3" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="H3" s="5" t="s">
         <v>28</v>
       </c>
+      <c r="I3" s="5" t="s">
+        <v>28</v>
+      </c>
       <c r="J3" s="18">
+        <v>0</v>
+      </c>
+      <c r="K3" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="K3" s="19" t="s">
-        <v>44</v>
-      </c>
       <c r="L3" s="22" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="M3" s="22" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="N3" s="22" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="O3" s="20" t="s">
-        <v>48</v>
-      </c>
-      <c r="P3" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q3" s="19" t="s">
-        <v>49</v>
-      </c>
-      <c r="R3" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="S3" s="17" t="s">
-        <v>37</v>
-      </c>
-      <c r="T3" s="16" t="s">
         <v>50</v>
       </c>
+      <c r="P3" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q3" s="19"/>
+      <c r="R3" s="17"/>
+      <c r="S3" s="17"/>
+      <c r="T3" s="16"/>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="G4" s="3" t="s">
+      <c r="A4" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="H4" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="I4" s="3" t="s">
+      <c r="C4" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="I4" s="5" t="s">
         <v>28</v>
       </c>
       <c r="J4" s="18">
         <v>46</v>
       </c>
       <c r="K4" s="19" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="L4" s="22" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="M4" s="22" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="N4" s="22" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="O4" s="20" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="P4" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="Q4" s="19"/>
       <c r="R4" s="17"/>
@@ -1221,19 +1222,19 @@
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>60</v>
+        <v>21</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>62</v>
+        <v>43</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>63</v>
@@ -1242,13 +1243,13 @@
         <v>64</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I5" s="5" t="s">
         <v>28</v>
       </c>
       <c r="J5" s="18">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="K5" s="19" t="s">
         <v>65</v>
@@ -1260,13 +1261,13 @@
         <v>67</v>
       </c>
       <c r="N5" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="O5" s="20" t="s">
         <v>68</v>
       </c>
-      <c r="O5" s="20" t="s">
-        <v>69</v>
-      </c>
       <c r="P5" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="Q5" s="19"/>
       <c r="R5" s="17"/>
@@ -1275,52 +1276,52 @@
     </row>
     <row r="6">
       <c r="A6" s="6" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="H6" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="I6" s="5" t="s">
         <v>71</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>28</v>
       </c>
       <c r="J6" s="18">
         <v>46</v>
       </c>
       <c r="K6" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="L6" s="22" t="s">
+        <v>73</v>
+      </c>
+      <c r="M6" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="N6" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="O6" s="20" t="s">
         <v>75</v>
       </c>
-      <c r="L6" s="22" t="s">
-        <v>76</v>
-      </c>
-      <c r="M6" s="22" t="s">
-        <v>77</v>
-      </c>
-      <c r="N6" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="O6" s="20" t="s">
-        <v>78</v>
-      </c>
       <c r="P6" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="Q6" s="19"/>
       <c r="R6" s="17"/>
@@ -1329,52 +1330,52 @@
     </row>
     <row r="7">
       <c r="A7" s="6" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>62</v>
+        <v>24</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="H7" s="5" t="s">
         <v>27</v>
       </c>
       <c r="I7" s="5" t="s">
-        <v>28</v>
+        <v>71</v>
       </c>
       <c r="J7" s="18">
         <v>100</v>
       </c>
       <c r="K7" s="19" t="s">
+        <v>79</v>
+      </c>
+      <c r="L7" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="M7" s="22" t="s">
         <v>81</v>
       </c>
-      <c r="L7" s="22" t="s">
+      <c r="N7" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="O7" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="M7" s="22" t="s">
-        <v>83</v>
-      </c>
-      <c r="N7" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="O7" s="20" t="s">
-        <v>84</v>
-      </c>
       <c r="P7" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="Q7" s="19"/>
       <c r="R7" s="17"/>
@@ -1382,53 +1383,53 @@
       <c r="T7" s="16"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="E8" s="6" t="s">
+      <c r="A8" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>86</v>
+      <c r="C8" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>28</v>
       </c>
       <c r="J8" s="18">
         <v>46</v>
       </c>
       <c r="K8" s="19" t="s">
+        <v>85</v>
+      </c>
+      <c r="L8" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="M8" s="22" t="s">
         <v>87</v>
       </c>
-      <c r="L8" s="22" t="s">
+      <c r="N8" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="O8" s="20" t="s">
         <v>88</v>
       </c>
-      <c r="M8" s="22" t="s">
-        <v>89</v>
-      </c>
-      <c r="N8" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="O8" s="20" t="s">
-        <v>90</v>
-      </c>
       <c r="P8" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="Q8" s="19"/>
       <c r="R8" s="17"/>
@@ -1436,53 +1437,53 @@
       <c r="T8" s="16"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="D9" s="6" t="s">
+      <c r="A9" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="J9" s="18">
+        <v>46</v>
+      </c>
+      <c r="K9" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>24</v>
-      </c>
-      <c r="F9" s="6" t="s">
+      <c r="L9" s="22" t="s">
         <v>92</v>
       </c>
-      <c r="G9" s="5" t="s">
+      <c r="M9" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="H9" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="I9" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="J9" s="18">
-        <v>100</v>
-      </c>
-      <c r="K9" s="19" t="s">
+      <c r="N9" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="O9" s="20" t="s">
         <v>94</v>
       </c>
-      <c r="L9" s="22" t="s">
-        <v>95</v>
-      </c>
-      <c r="M9" s="22" t="s">
-        <v>96</v>
-      </c>
-      <c r="N9" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="O9" s="20" t="s">
-        <v>97</v>
-      </c>
       <c r="P9" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="Q9" s="19"/>
       <c r="R9" s="17"/>
@@ -1491,52 +1492,52 @@
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>39</v>
+        <v>76</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>98</v>
+        <v>44</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="H10" s="7" t="s">
-        <v>43</v>
+        <v>27</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>28</v>
       </c>
       <c r="J10" s="18">
-        <v>46</v>
+        <v>100</v>
       </c>
       <c r="K10" s="19" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="L10" s="22" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="M10" s="22" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="N10" s="22" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="O10" s="20" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="P10" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="Q10" s="19"/>
       <c r="R10" s="17"/>
@@ -1545,52 +1546,52 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>24</v>
+        <v>100</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>28</v>
+        <v>103</v>
       </c>
       <c r="J11" s="18">
         <v>46</v>
       </c>
       <c r="K11" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="L11" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="M11" s="22" t="s">
         <v>106</v>
       </c>
-      <c r="L11" s="22" t="s">
+      <c r="N11" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="O11" s="20" t="s">
         <v>107</v>
       </c>
-      <c r="M11" s="22" t="s">
-        <v>108</v>
-      </c>
-      <c r="N11" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="O11" s="20" t="s">
-        <v>109</v>
-      </c>
       <c r="P11" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="Q11" s="19"/>
       <c r="R11" s="17"/>
@@ -1599,25 +1600,25 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>91</v>
+        <v>23</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>62</v>
+        <v>24</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>63</v>
+        <v>108</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>27</v>
@@ -1629,22 +1630,22 @@
         <v>100</v>
       </c>
       <c r="K12" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="L12" s="22" t="s">
         <v>111</v>
       </c>
-      <c r="L12" s="22" t="s">
+      <c r="M12" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="M12" s="22" t="s">
+      <c r="N12" s="22" t="s">
         <v>113</v>
-      </c>
-      <c r="N12" s="22" t="s">
-        <v>68</v>
       </c>
       <c r="O12" s="20" t="s">
         <v>114</v>
       </c>
       <c r="P12" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="Q12" s="19"/>
       <c r="R12" s="17"/>
@@ -1653,52 +1654,52 @@
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>71</v>
+        <v>22</v>
       </c>
       <c r="D13" s="8" t="s">
-        <v>91</v>
+        <v>23</v>
       </c>
       <c r="E13" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F13" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="G13" s="7" t="s">
         <v>116</v>
       </c>
-      <c r="G13" s="7" t="s">
-        <v>117</v>
-      </c>
       <c r="H13" s="7" t="s">
-        <v>43</v>
+        <v>58</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>118</v>
+        <v>28</v>
       </c>
       <c r="J13" s="18">
         <v>46</v>
       </c>
       <c r="K13" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="L13" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="M13" s="22" t="s">
         <v>119</v>
       </c>
-      <c r="L13" s="22" t="s">
+      <c r="N13" s="22" t="s">
+        <v>49</v>
+      </c>
+      <c r="O13" s="20" t="s">
         <v>120</v>
       </c>
-      <c r="M13" s="22" t="s">
-        <v>121</v>
-      </c>
-      <c r="N13" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="O13" s="20" t="s">
-        <v>122</v>
-      </c>
       <c r="P13" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="Q13" s="19"/>
       <c r="R13" s="17"/>
@@ -1707,25 +1708,25 @@
     </row>
     <row r="14">
       <c r="A14" s="8" t="s">
-        <v>71</v>
+        <v>53</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>71</v>
+        <v>22</v>
       </c>
       <c r="D14" s="8" t="s">
         <v>23</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>27</v>
@@ -1737,22 +1738,22 @@
         <v>100</v>
       </c>
       <c r="K14" s="19" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="L14" s="22" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
       <c r="M14" s="22" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="N14" s="22" t="s">
-        <v>128</v>
+        <v>49</v>
       </c>
       <c r="O14" s="20" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="P14" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="Q14" s="19"/>
       <c r="R14" s="17"/>
@@ -1760,53 +1761,53 @@
       <c r="T14" s="16"/>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="B15" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="8" t="s">
+      <c r="A15" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="D15" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E15" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="F15" s="8" t="s">
-        <v>130</v>
-      </c>
-      <c r="G15" s="7" t="s">
-        <v>131</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="I15" s="7" t="s">
-        <v>28</v>
+      <c r="E15" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F15" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="G15" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>125</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>103</v>
       </c>
       <c r="J15" s="18">
-        <v>46</v>
+        <v>1</v>
       </c>
       <c r="K15" s="19" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="L15" s="22" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="M15" s="22" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="N15" s="22" t="s">
-        <v>68</v>
+        <v>49</v>
       </c>
       <c r="O15" s="20" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="P15" s="10" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="Q15" s="19"/>
       <c r="R15" s="17"/>
@@ -1814,89 +1815,97 @@
       <c r="T15" s="16"/>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="B16" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="C16" s="8" t="s">
+      <c r="A16" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="E16" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="F16" s="8" t="s">
+      <c r="B16" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="17" t="s">
+        <v>42</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="F16" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="G16" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="G16" s="7" t="s">
+      <c r="H16" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="I16" s="21" t="s">
+        <v>28</v>
+      </c>
+      <c r="J16" s="18">
+        <v>46</v>
+      </c>
+      <c r="K16" s="19" t="s">
         <v>131</v>
       </c>
-      <c r="H16" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="I16" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="J16" s="18">
-        <v>100</v>
-      </c>
-      <c r="K16" s="19" t="s">
+      <c r="L16" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="M16" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="N16" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="O16" s="20" t="s">
+        <v>135</v>
+      </c>
+      <c r="P16" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="L16" s="22" t="s">
-        <v>133</v>
-      </c>
-      <c r="M16" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="N16" s="22" t="s">
-        <v>68</v>
-      </c>
-      <c r="O16" s="20" t="s">
+      <c r="Q16" s="19" t="s">
         <v>137</v>
       </c>
-      <c r="P16" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q16" s="19"/>
-      <c r="R16" s="17"/>
-      <c r="S16" s="17"/>
-      <c r="T16" s="16"/>
+      <c r="R16" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="S16" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="T16" s="16" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>60</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>138</v>
-      </c>
-      <c r="D17" s="10" t="s">
+      <c r="A17" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="17" t="s">
         <v>23</v>
       </c>
-      <c r="E17" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="F17" s="10" t="s">
-        <v>63</v>
-      </c>
-      <c r="G17" s="9" t="s">
+      <c r="E17" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="F17" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="G17" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="I17" s="9" t="s">
-        <v>118</v>
+      <c r="H17" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="I17" s="21" t="s">
+        <v>28</v>
       </c>
       <c r="J17" s="18">
-        <v>1</v>
+        <v>46</v>
       </c>
       <c r="K17" s="19" t="s">
         <v>141</v>
@@ -1908,18 +1917,26 @@
         <v>143</v>
       </c>
       <c r="N17" s="22" t="s">
-        <v>68</v>
+        <v>144</v>
       </c>
       <c r="O17" s="20" t="s">
-        <v>144</v>
-      </c>
-      <c r="P17" s="10" t="s">
-        <v>58</v>
-      </c>
-      <c r="Q17" s="19"/>
-      <c r="R17" s="17"/>
-      <c r="S17" s="17"/>
-      <c r="T17" s="16"/>
+        <v>145</v>
+      </c>
+      <c r="P17" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="Q17" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="R17" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="S17" s="17" t="s">
+        <v>37</v>
+      </c>
+      <c r="T17" s="16" t="s">
+        <v>147</v>
+      </c>
     </row>
   </sheetData>
   <pageSetup orientation="landscape" paperSize="9"/>

</xml_diff>